<commit_message>
5/12: 버튼 4-tier, Invoice 개선, vehicle per_day, Edit picker sticky, Financials 최상단, agent 비활성화 차단
- 버튼 4-tier 체계 확정 (Primary/Edit/Utility/Destructive) — 15개 파일 적용
- Invoice: SVG 아이콘 통일, Copy Link 조건부 숨김, Send Invoice 이메일 버튼
- canEdit = !!currentAdminId (assigned_admin_id 게이트 제거)
- Health Screening 업로드 파싱: 성별을 상품명에 합쳐 독립 product 분리
- 카탈로그 3차 partner pills + subcategory 섹션 뷰
- 상품 삭제 이름 입력 확인 모달
- vehicle per_day: daysBetween early-return + daysLive live variable (호텔과 동일 패턴)
- Edit Selected Products: 자동스크롤(rAF) + sticky picker + 드롭다운 upward
- completed 케이스 Financials 최상단: flex flex-col + CSS order
- agent 비활성화 3-layer: login signOut + AgentOnboardingGuard + /deactivated 전용 페이지

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/products_master_v21.xlsx
+++ b/data/products_master_v21.xlsx
@@ -1,22 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04CEA6B1-61BC-40FC-A781-54A6693B7F27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="K-Medical" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="K-Beauty" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="K-Wellness" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="K-Starcation" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="K-Education" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="Subpackage" state="visible" r:id="rId9"/>
+    <sheet name="K-Medical" sheetId="1" r:id="rId1"/>
+    <sheet name="K-Beauty" sheetId="2" r:id="rId2"/>
+    <sheet name="K-Wellness" sheetId="3" r:id="rId3"/>
+    <sheet name="K-Starcation" sheetId="4" r:id="rId4"/>
+    <sheet name="K-Education" sheetId="5" r:id="rId5"/>
+    <sheet name="Subpackage" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9560" uniqueCount="1578">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9450" uniqueCount="1578">
   <si>
     <t>product_number</t>
   </si>
@@ -138,7 +142,7 @@
     <t>days</t>
   </si>
   <si>
-    <t xml:space="preserve">* Heart &amp; Brain Premium + Additional Tests
+    <t>* Heart &amp; Brain Premium + Additional Tests
 * An advanced program developed for early detection of cancer and cardio-cerebrovascular diseases, carefully tailored to each individual's medical history and needs
 * Recommended for ages 50+</t>
   </si>
@@ -173,7 +177,7 @@
     <t>VIP Premium</t>
   </si>
   <si>
-    <t xml:space="preserve">* Heart &amp; Brain Premium + Additional Tests
+    <t>* Heart &amp; Brain Premium + Additional Tests
 * A premium all-in-one screening program offering a comprehensive health evaluation
 * Recommended for ages 50+</t>
   </si>
@@ -196,7 +200,7 @@
     <t>USD</t>
   </si>
   <si>
-    <t xml:space="preserve">Common : Fundus Photography ❖Age ≥50: including Audiometry, excluding Hepatitis A
+    <t>Common : Fundus Photography ❖Age ≥50: including Audiometry, excluding Hepatitis A
 M : Prostate Tumor Marker
 F : Gynecologic Examination &amp; Consultation, Ovarian Tumor Marker, Cervical Cytologic 
       Test(PAP Smear), Mammography</t>
@@ -235,7 +239,7 @@
     <t>Basic Intensive</t>
   </si>
   <si>
-    <t xml:space="preserve">Includes International Basic +
+    <t>Includes International Basic +
 Thyroid Ultrasonography / Pelvic Ultrasonography
 Breast Ultrasonography / Low dose Chest CT
 HPV(Human Papilloma Virus) / Bone densitometry / Vitamin D
@@ -258,7 +262,7 @@
     <t>Premium S</t>
   </si>
   <si>
-    <t xml:space="preserve">Includes International Basic +
+    <t>Includes International Basic +
 Pre-medical consultation / Brain MRI·MRA, Colonoscopy under conscious sedation
 Thyroid Ultrasonography / Carotid Ultrasonography
 Echocardiography / Coronary artery 3D CT / Low dose Chest CT
@@ -276,7 +280,7 @@
     <t>Premium P</t>
   </si>
   <si>
-    <t xml:space="preserve">Includes International Marian S +
+    <t>Includes International Marian S +
 Optical CT(Retina / Glaucoma)
 Detailed Blood test(Parathyroid hormone, Factor of Arteriosclerosis)
 Tumor marker(Thyroid)
@@ -298,7 +302,7 @@
     <t>Essential</t>
   </si>
   <si>
-    <t xml:space="preserve">•Gastroscopy Under Conscious Sedation     •Abdominal Ultrasonography
+    <t>•Gastroscopy Under Conscious Sedation     •Abdominal Ultrasonography
 •Blood Pressure     •Electrocardiogram
 •Chest X-ray (Front/Lateral)    •Ophthalmic Exam
 •Urine Test    •Audiometry Test    •Body Measurement    •Dental Assessment
@@ -325,7 +329,7 @@
     <t>Platinum</t>
   </si>
   <si>
-    <t xml:space="preserve">Extensive and Detailed Check-up Program Including Cancer &amp; Heart Program and Brain MR Male
+    <t>Extensive and Detailed Check-up Program Including Cancer &amp; Heart Program and Brain MR Male
 Essential +
 •Brain MRA &amp; MRI •Abdominal &amp; Pelvic CT •Coronary CT •Echocardiography •Treadmill Test
 •Arterial Stiffness and Peripheral Artery Stenosis •Dental X-ray
@@ -376,14 +380,14 @@
     <t>minutes</t>
   </si>
   <si>
-    <t xml:space="preserve">* Vaginal rejuvenation laser (600 shots) + tightening treatment + sensory enhancement injection
+    <t>* Vaginal rejuvenation laser (600 shots) + tightening treatment + sensory enhancement injection
 * Labia whitening &amp; moisturizing treatment
 * Premium IV nutrition: high-dose amino acids, B-complex, vitamin C, garlic injection
 * Volume filler 10cc
 * Comprehensive women's health screening: hormone panel, pelvic ultrasound (uterus/ovaries/bladder), cancer markers, STD panel</t>
   </si>
   <si>
-    <t xml:space="preserve">* Dedicated women's health clinic specializing in VIP feminine rejuvenation
+    <t>* Dedicated women's health clinic specializing in VIP feminine rejuvenation
 * Comprehensive programs combining aesthetic, hormonal, and preventive care
 * Female doctors available upon request</t>
   </si>
@@ -400,7 +404,7 @@
     <t>VIP Anti-Aging</t>
   </si>
   <si>
-    <t xml:space="preserve">* All inclusions of Premium Rejuvenation Package
+    <t>* All inclusions of Premium Rejuvenation Package
 * Volume filler 15cc
 * Stem cell ovarian anti-aging injection for hormonal rejuvenation</t>
   </si>
@@ -411,7 +415,7 @@
     <t>Royal Total Luxury</t>
   </si>
   <si>
-    <t xml:space="preserve">* All inclusions of VIP Anti-Aging Package
+    <t>* All inclusions of VIP Anti-Aging Package
 * Volume filler 25cc
 * External volumizing program (Juvelook Volume)</t>
   </si>
@@ -440,7 +444,7 @@
     <t>months</t>
   </si>
   <si>
-    <t xml:space="preserve">* Dentium SuperLine implant fixture (South Korean, premium quality)
+    <t>* Dentium SuperLine implant fixture (South Korean, premium quality)
 * Custom abutment + zirconia crown
 * Bone graft included
 * Fixture: titanium screw anchored into jawbone
@@ -448,7 +452,7 @@
 * Treatment duration: 3–6 months per implant</t>
   </si>
   <si>
-    <t xml:space="preserve">* Premium implant packages combining Korean and Swiss-brand systems
+    <t>* Premium implant packages combining Korean and Swiss-brand systems
 * Bone graft included in all implant packages — no hidden add-on costs
 * Highly competitive pricing compared to Western dental clinics</t>
   </si>
@@ -462,7 +466,7 @@
     <t>Straumann</t>
   </si>
   <si>
-    <t xml:space="preserve">* Straumann implant fixture (Swiss, globally recognized premium brand)
+    <t>* Straumann implant fixture (Swiss, globally recognized premium brand)
 * Custom abutment + zirconia crown
 * Bone graft included
 * Fixture: titanium screw anchored into jawbone
@@ -479,7 +483,7 @@
     <t>8–12</t>
   </si>
   <si>
-    <t xml:space="preserve">* 7 Dentium SuperLine implant fixtures + 7 custom abutments + 7 zirconia crowns
+    <t>* 7 Dentium SuperLine implant fixtures + 7 custom abutments + 7 zirconia crowns
 * Bone graft included for all 7 implants
 * 5 bridge connector teeth (pontics)
 * Full arch (upper or lower jaw) implant restoration
@@ -495,7 +499,7 @@
     <t>Sinus Lift</t>
   </si>
   <si>
-    <t xml:space="preserve">* Elevation of the maxillary sinus membrane to create space for implant placement in the upper molar region
+    <t>* Elevation of the maxillary sinus membrane to create space for implant placement in the upper molar region
 * Required when jawbone height is insufficient for direct implant placement
 * Bone graft performed simultaneously during the procedure
 * Optional add-on to dental implant treatment</t>
@@ -2874,13 +2878,13 @@
     <t>Korea Grand Sale Shopping Festival</t>
   </si>
   <si>
-    <t xml:space="preserve">* Korea's premier annual shopping, culture, and tourism festival
+    <t>* Korea's premier annual shopping, culture, and tourism festival
 * Welcome coupon book, K-theme zone experiences, photo zones &amp; lucky draw
 * AI-powered shopping recommendations and K-Shopping Cart event
 * Covers: air/transport, shopping, accommodation, dining, beauty, health, and concierge services</t>
   </si>
   <si>
-    <t xml:space="preserve">* Nation's largest multi-sector shopping &amp; tourism festival with K-cultural experiences
+    <t>* Nation's largest multi-sector shopping &amp; tourism festival with K-cultural experiences
 * Exclusive foreign-visitor welcome coupons and themed activities included</t>
   </si>
   <si>
@@ -2908,7 +2912,7 @@
     <t>Premium Optical &amp; Eyewear</t>
   </si>
   <si>
-    <t xml:space="preserve">* Korea's largest Lindberg dealer — premium international designer eyewear
+    <t>* Korea's largest Lindberg dealer — premium international designer eyewear
 * State-of-the-art digital lens fitting and advanced 3D diagnostic equipment
 * Highly trained optometrists with precision fitting systems
 * Branches: Dogok, Samsung Medical Center, Apgujeong, KINTEX, Pangyo, Cheonho, Express Bus Terminal, Apgujeong Rodeo, Gwanggyo, Yeouido, Myeongdong, Jamsil</t>
@@ -2938,7 +2942,7 @@
     <t>K-Beauty Shopping</t>
   </si>
   <si>
-    <t xml:space="preserve">* Korea's first and largest health &amp; beauty retail chain
+    <t>* Korea's first and largest health &amp; beauty retail chain
 * Curated selection of K-cosmetics, health supplements, beauty tools, and lifestyle products
 * Mix of Korean indie brands and global favorites under one roof</t>
   </si>
@@ -2961,7 +2965,7 @@
     <t>K-Stationery &amp; Lifestyle Shopping</t>
   </si>
   <si>
-    <t xml:space="preserve">* Korea's first design-focused stationery and lifestyle brand
+    <t>* Korea's first design-focused stationery and lifestyle brand
 * Pioneered the transformation of stationery into a design-driven lifestyle category
 * Stylish stationery, planners, home goods, and K-culture merchandise</t>
   </si>
@@ -2990,13 +2994,13 @@
     <t>K-POP Demon Hunters Tour</t>
   </si>
   <si>
-    <t xml:space="preserve">* Immersive mission-based XR/AR K-POP adventure through iconic Seoul landmarks
+    <t>* Immersive mission-based XR/AR K-POP adventure through iconic Seoul landmarks
 * Gyeongbokgung → Bukchon/Seochon → Myeongdong → VAN Entertainment DIY Workshop → Naksan Park → souvenir shopping
 * Includes: 1 van, English guide, professional photographer, and lunch
 * Min. 2 / max. 6–7 persons per group</t>
   </si>
   <si>
-    <t xml:space="preserve">* K-POP Demon Hunters world brought to life with cutting-edge XR/AR technology
+    <t>* K-POP Demon Hunters world brought to life with cutting-edge XR/AR technology
 * Professional photographer and English guide included; mission-style immersive format</t>
   </si>
   <si>
@@ -3021,12 +3025,12 @@
     <t>SBS Inkigayo K-POP Concert Package</t>
   </si>
   <si>
-    <t xml:space="preserve">* Live taping ticket for SBS Inkigayo at SBS Public Hall (every Sunday)
+    <t>* Live taping ticket for SBS Inkigayo at SBS Public Hall (every Sunday)
 * Walking tour with monthly-changing itinerary + transportation to SBS Public Hall
 * Passport required; exclusive to foreign visitors</t>
   </si>
   <si>
-    <t xml:space="preserve">* Attend a real K-POP music show taping (SBS Inkigayo) every Sunday
+    <t>* Attend a real K-POP music show taping (SBS Inkigayo) every Sunday
 * Exclusive foreign-visitor package: walking tour + live show entry</t>
   </si>
   <si>
@@ -3045,7 +3049,7 @@
     <t>K-Drama Filming Location Tour (Seoul)</t>
   </si>
   <si>
-    <t xml:space="preserve">* Descendants of the Sun, Guardian: The Lonely and Great God, My Love From the Star filming locations
+    <t>* Descendants of the Sun, Guardian: The Lonely and Great God, My Love From the Star filming locations
 * Route: Songdo Dalkomm Coffee → Songdo Central Park → Deoksugung → Hakrim Coffee → N Seoul Tower
 * Lunch at BBQ restaurant (Guardian filming site) included; private guide throughout</t>
   </si>
@@ -3065,7 +3069,7 @@
     <t>K-Drama Filming Location Tour (Jeju)</t>
   </si>
   <si>
-    <t xml:space="preserve">* Welcome to Samdal-ri, Extraordinary Attorney Woo, When Life Gives You Tangerines — Jeju filming locations
+    <t>* Welcome to Samdal-ri, Extraordinary Attorney Woo, When Life Gives You Tangerines — Jeju filming locations
 * Route A: Gwaneumsa Temple, Secret Forest Andol-oreum, Gwangchigi Beach, Seongsan Ilchulbong, Seongiwpean Bakery
 * Route B: Dodubong Peak, Rainbow Coastal Road, Iho Taewooja Horse Lighthouses, Myeongwol Elementary School, Changsindo
 * Private guide-accompanied tour; vehicle included; meals at guest discretion</t>
@@ -3089,7 +3093,7 @@
     <t>Squid Game Tour (Incheon)</t>
   </si>
   <si>
-    <t xml:space="preserve">* Visit Gyodong Elementary — a real Squid Game filming location
+    <t>* Visit Gyodong Elementary — a real Squid Game filming location
 * On-screen challenges: dalgona carving and punch machine
 * Retro "lunchbox" meal as seen on screen + sea-view monorail loop
 * Archery Café at Wolmi Island + Songdo Central Park mission game
@@ -3111,12 +3115,12 @@
     <t>K-POP Idol VIP Experience</t>
   </si>
   <si>
-    <t xml:space="preserve">* VIP-only private K-POP idol experience — limited to 4 participants per day
+    <t>* VIP-only private K-POP idol experience — limited to 4 participants per day
 * K-POP idol dance training + vocal training → idol concept makeup → idol concept photo shoot
 * Lunch (Korean cuisine) included</t>
   </si>
   <si>
-    <t xml:space="preserve">* Ultra-exclusive private K-POP program: max. 4 guests per day
+    <t>* Ultra-exclusive private K-POP program: max. 4 guests per day
 * Full idol training experience — dance, vocals, makeup, and professional photo shoot</t>
   </si>
   <si>
@@ -3132,7 +3136,7 @@
     <t>K-POP One Day Dance Lesson</t>
   </si>
   <si>
-    <t xml:space="preserve">* Private K-POP one-day dance class tailored to group skill level and purpose
+    <t>* Private K-POP one-day dance class tailored to group skill level and purpose
 * Lesson counseling → instructor assignment → lesson start
 * Small-group format with professional choreography instructor; studio in Seoul</t>
   </si>
@@ -3161,7 +3165,7 @@
     <t>1 Person</t>
   </si>
   <si>
-    <t xml:space="preserve">* 1-on-1 styling session with a professional Korean fashion stylist
+    <t>* 1-on-1 styling session with a professional Korean fashion stylist
 * 6–7 curated outfit recommendations per hour from popular Korean fashion brands
 * Final purchase decisions entirely at the guest discretion; Seoul Gangnam area</t>
   </si>
@@ -3184,12 +3188,12 @@
     <t>K-Beauty Makeup &amp; Hair Styling</t>
   </si>
   <si>
-    <t xml:space="preserve">* Professional K-Beauty styling at studios where Korean celebrities prepare for performances
+    <t>* Professional K-Beauty styling at studios where Korean celebrities prepare for performances
 * Makeup + Hair Styling + Photoshoot package
 * Studio in Gangnam Cheongdam-dong, Dosan Park area; near Supreme, Louis Vuitton, Stussy</t>
   </si>
   <si>
-    <t xml:space="preserve">* Get styled at the same salon Korean entertainment stars use before shows
+    <t>* Get styled at the same salon Korean entertainment stars use before shows
 * Complete K-Beauty transformation: hair, makeup, and professional photoshoot</t>
   </si>
   <si>
@@ -3208,7 +3212,7 @@
     <t>Master Style Consulting</t>
   </si>
   <si>
-    <t xml:space="preserve">* I Style Consulting: professional image consulting — hair, makeup, personal color, and body type analysis
+    <t>* I Style Consulting: professional image consulting — hair, makeup, personal color, and body type analysis
 * Fit Style Consulting: advanced body-type fit styling based on data from 15,000+ measurements
 * In-person analysis plus practical shopping guidance; combined I Style + Fit Style package (300 min)</t>
   </si>
@@ -3228,7 +3232,7 @@
     <t>VIP Private Consulting</t>
   </si>
   <si>
-    <t xml:space="preserve">* Ultra-premium VIP offline service by prior inquiry only
+    <t>* Ultra-premium VIP offline service by prior inquiry only
 * Comprehensive consulting: hair, makeup, fashion, and signature style design
 * 1:1 customized analysis and style proposal; inquiries via email only</t>
   </si>
@@ -3251,7 +3255,7 @@
     <t>VIP Offline Consulting</t>
   </si>
   <si>
-    <t xml:space="preserve">* VIP private consulting by a team of specialist consultants
+    <t>* VIP private consulting by a team of specialist consultants
 * Includes: Beauty, Fashion, Hair, and Makeup consulting
 * KakaoTalk channel inquiries accepted</t>
   </si>
@@ -3274,7 +3278,7 @@
     <t>Master Premium Personal Color Diagnosis</t>
   </si>
   <si>
-    <t xml:space="preserve">* 25-type detailed seasonal tone color draping analysis
+    <t>* 25-type detailed seasonal tone color draping analysis
 * Color cosmetics, fashion style, accessories, perfume, glasses/lens, and nail recommendations
 * Body structure analysis + strategic fashion coaching + signature image consulting</t>
   </si>
@@ -3294,7 +3298,7 @@
     <t>Palette Premium Personal Color Diagnosis</t>
   </si>
   <si>
-    <t xml:space="preserve">* In-depth personal color diagnosis after body color analysis
+    <t>* In-depth personal color diagnosis after body color analysis
 * Hair, jewelry, and lens color recommendations
 * Face zone mini analysis + fashion coaching + perfume, necklace, earring, ring, and watch recommendations</t>
   </si>
@@ -3317,13 +3321,13 @@
     <t>Seoul City Tour</t>
   </si>
   <si>
-    <t xml:space="preserve">* VIP Special Full-Day Seoul City Tour — min. 4 persons / 09:00–17:30
+    <t>* VIP Special Full-Day Seoul City Tour — min. 4 persons / 09:00–17:30
 * Hotel → City Hall/Gwanghwamun/Cheonggyecheon → Royal Guard Ceremony → Gyeongbokgung → National Folk Museum
 * → Amethyst/Ginseng Center → N Seoul Tower → Lunch → Changdeokgung → Insadong → Han River Cruise → Hotel
 * Private vehicle, professional English guide, and lunch included</t>
   </si>
   <si>
-    <t xml:space="preserve">* Full-day premium private Seoul tour covering history, culture, and scenic landmarks
+    <t>* Full-day premium private Seoul tour covering history, culture, and scenic landmarks
 * Private vehicle + English guide + lunch all included</t>
   </si>
   <si>
@@ -3345,7 +3349,7 @@
     <t>Seoul City Night Tour</t>
   </si>
   <si>
-    <t xml:space="preserve">* Bamdokkaebi (Night Goblin) night driving tour of Seoul illuminated landmarks
+    <t>* Bamdokkaebi (Night Goblin) night driving tour of Seoul illuminated landmarks
 * Route: Gwanghwamun Square → Cheonggyecheon → DDP → N Seoul Tower → Han River Park → Banpo Moonbow Fountain → Itaewon
 * English-speaking guide; exclusive to foreign visitors; passport required</t>
   </si>
@@ -3374,12 +3378,12 @@
     <t>Islamic Seoul City Tour</t>
   </si>
   <si>
-    <t xml:space="preserve">* Muslim-only private Seoul city tour with halal meals and dedicated prayer time
+    <t>* Muslim-only private Seoul city tour with halal meals and dedicated prayer time
 * Route: Hotel → Hanbok → Royal Guard Ceremony → Gyeongbokgung → N Seoul Tower → Itaewon Mosque → Halal Lunch → Prayer Time → Bukchon Village → Dongdaemun Market → Gwangjang Market → Myeongdong
 * Includes: private vehicle, halal lunch, entrance fees, Arabic/English guide</t>
   </si>
   <si>
-    <t xml:space="preserve">* Fully Muslim-friendly Seoul tour with halal dining and prayer time arranged
+    <t>* Fully Muslim-friendly Seoul tour with halal dining and prayer time arranged
 * Arabic and English-speaking guide; private vehicle included</t>
   </si>
   <si>
@@ -3395,12 +3399,12 @@
     <t>DMZ + NLL Tour</t>
   </si>
   <si>
-    <t xml:space="preserve">* VIP Private DMZ + NLL Tour — min. 4 persons / 07:00–17:30
+    <t>* VIP Private DMZ + NLL Tour — min. 4 persons / 07:00–17:30
 * Route: Hotel → Imjingak → Unification Bridge → Passport check → DMZ Theater &amp; Exhibition → 3rd Tunnel → Dora Observatory → Unification Village → Lunch → Ganghwa Island coastal fence → Ganghwa Peace Observatory → Hotel
 * Private vehicle and professional guide; lunch included</t>
   </si>
   <si>
-    <t xml:space="preserve">* Exclusive VIP tour to the Korean DMZ and NLL — Korea's most politically significant restricted zones
+    <t>* Exclusive VIP tour to the Korean DMZ and NLL — Korea's most politically significant restricted zones
 * Includes 3rd Tunnel, Dora Observatory, and Ganghwa Island NLL area</t>
   </si>
   <si>
@@ -3419,7 +3423,7 @@
     <t>Islamic Nami Island Tour</t>
   </si>
   <si>
-    <t xml:space="preserve">* Muslim-only private tour to Nami Island and Garden of Morning Calm
+    <t>* Muslim-only private tour to Nami Island and Garden of Morning Calm
 * Route: Hotel → Nami Island → Halal lunch → Prayer time → Garden of Morning Calm → Hotel or Myeongdong
 * Includes: private vehicle, halal lunch, Arabic/English guide</t>
   </si>
@@ -3442,14 +3446,14 @@
     <t>Jeju Island Private Tour</t>
   </si>
   <si>
-    <t xml:space="preserve">* Private 3-day Jeju Island tour with Grand Hyatt Jeju accommodation
+    <t>* Private 3-day Jeju Island tour with Grand Hyatt Jeju accommodation
 * Inclusions: round-trip airfare, Grand Hyatt Jeju, private vehicle + driver (Solati 4–10P / Combi Bus 11P+)
 * Meals per itinerary (breakfast, lunch, one dinner daily)
 * Admission: Pacific Marina Yacht, Hwansang Forest Gotjawal Park + foot bath, full-body massage
 * Travel insurance included; itinerary customizable</t>
   </si>
   <si>
-    <t xml:space="preserve">* Fully inclusive luxury 3-day Jeju tour: Grand Hyatt, private driver, yacht, and spa massage
+    <t>* Fully inclusive luxury 3-day Jeju tour: Grand Hyatt, private driver, yacht, and spa massage
 * Travel insurance and all admission fees included</t>
   </si>
   <si>
@@ -3468,13 +3472,13 @@
     <t>Jeju Island Golf Tour</t>
   </si>
   <si>
-    <t xml:space="preserve">* Premium 3-day Jeju golf tour with Blackstone Villa Suite accommodation
+    <t>* Premium 3-day Jeju golf tour with Blackstone Villa Suite accommodation
 * 3 rounds of 18-hole golf: 2 rounds at Blackstone CC + 1 round at Elysian CC
 * Both courses ranked in Asia Top 100; 2 nights private villa; private vehicle
 * Meals not included</t>
   </si>
   <si>
-    <t xml:space="preserve">* Play three rounds at Jeju's top-ranked courses: Blackstone CC and Elysian CC (Asia Top 100)
+    <t>* Play three rounds at Jeju's top-ranked courses: Blackstone CC and Elysian CC (Asia Top 100)
 * Blackstone Villa Suite accommodation with private vehicle</t>
   </si>
   <si>
@@ -3496,7 +3500,7 @@
     <t>Gyeongbuk Tourpass</t>
   </si>
   <si>
-    <t xml:space="preserve">* Free-pass ticket for major paid attractions across Gyeongsangbuk-do
+    <t>* Free-pass ticket for major paid attractions across Gyeongsangbuk-do
 * Single barcode grants 24/48/72-hour unlimited access to multiple attractions
 * Covers: Gyeongju, Pohang, Ulleungdo, and partner cafés; various route options</t>
   </si>
@@ -3522,12 +3526,12 @@
     <t>Busan One-Night Cruise</t>
   </si>
   <si>
-    <t xml:space="preserve">* Busan Fanstar one-night luxury cruise departing from Busan Port
+    <t>* Busan Fanstar one-night luxury cruise departing from Busan Port
 * Inclusions: Panstar Bridge Tour, onboard dinner buffet, live performances and events, fireworks
 * Breakfast included on return; operates every Saturday (rotating routes)</t>
   </si>
   <si>
-    <t xml:space="preserve">* Overnight luxury cruise from Busan with fireworks, live shows, and scenic Korea Strait seascape
+    <t>* Overnight luxury cruise from Busan with fireworks, live shows, and scenic Korea Strait seascape
 * All-inclusive: dinner buffet, breakfast, entertainment, and duty-free shopping</t>
   </si>
   <si>
@@ -3549,12 +3553,12 @@
     <t>Grand Tour of Korea by Rail Cruise</t>
   </si>
   <si>
-    <t xml:space="preserve">* 3-day nationwide AURA rail cruise across Korea's most scenic regions
+    <t>* 3-day nationwide AURA rail cruise across Korea's most scenic regions
 * Route: Suncheon → Yeosu → Busan → Gyeongju → Jeongdongjin → Donghae → Seoul
 * All-inclusive: train fare, connecting buses, onboard accommodation, all meals &amp; snacks, beverages, entrance &amp; activity fees, onboard events</t>
   </si>
   <si>
-    <t xml:space="preserve">* All-inclusive 3-day luxury rail journey through Korea's most beautiful scenic regions
+    <t>* All-inclusive 3-day luxury rail journey through Korea's most beautiful scenic regions
 * Accommodation, meals, entrance fees, and entertainment all included on Rail Cruise Haerang</t>
   </si>
   <si>
@@ -3588,7 +3592,7 @@
     <t>1–2</t>
   </si>
   <si>
-    <t xml:space="preserve">* MONA Yongpyong Resort — Korea's largest ski resort; 28 slopes, 14 lifts, 13 FIS-certified runs
+    <t>* MONA Yongpyong Resort — Korea's largest ski resort; 28 slopes, 14 lifts, 13 FIS-certified runs
 * Rental: ski/snowboard equipment and clothing; lift ticket included
 * Lesson: professional instructor (group or private); separate pricing</t>
   </si>
@@ -3626,7 +3630,7 @@
     <t>High 1 Resort Ski Package</t>
   </si>
   <si>
-    <t xml:space="preserve">* High 1 Resort — 15 FIS-certified slopes, 5 lifts, 3 gondolas; sleigh riding also available
+    <t>* High 1 Resort — 15 FIS-certified slopes, 5 lifts, 3 gondolas; sleigh riding also available
 * Rental: ski/snowboard equipment and clothing; lift ticket included
 * Lesson: professional instructor available</t>
   </si>
@@ -3661,7 +3665,7 @@
     <t>Vivaldi Park Ski Package</t>
   </si>
   <si>
-    <t xml:space="preserve">* Vivaldi Park Resort — 13 slopes, 10 lifts
+    <t>* Vivaldi Park Resort — 13 slopes, 10 lifts
 * Rental: ski/snowboard equipment and clothing; lift ticket included
 * Lesson: professional instructor available</t>
   </si>
@@ -3690,7 +3694,7 @@
     <t>Konjiam Resort Ski Package</t>
   </si>
   <si>
-    <t xml:space="preserve">* Konjiam Resort — 9 slopes, 5 lifts; closest major ski resort to Seoul
+    <t>* Konjiam Resort — 9 slopes, 5 lifts; closest major ski resort to Seoul
 * Rental: ski/snowboard equipment and clothing; lift ticket included
 * Lesson: professional instructor available</t>
   </si>
@@ -3719,7 +3723,7 @@
     <t>Middle Season Pass</t>
   </si>
   <si>
-    <t xml:space="preserve">* Caribbean Bay — Korea's premier water park at Everland Resort
+    <t>* Caribbean Bay — Korea's premier water park at Everland Resort
 * Caribbean-themed: wave pool, diving pool, surfing ride, and slides
 * Seasonal pricing (Middle / High / Gold season)</t>
   </si>
@@ -3757,7 +3761,7 @@
     <t>Mid-Summer Pass</t>
   </si>
   <si>
-    <t xml:space="preserve">* Ocean World — large-scale water park at Vivaldi Park Resort
+    <t>* Ocean World — large-scale water park at Vivaldi Park Resort
 * Ancient Egyptian theme: wave pool, mega slides, and adventure zones
 * Seasonal pricing (Mid-Summer / Hot Summer)</t>
   </si>
@@ -3792,7 +3796,7 @@
     <t>Normal Season (6h)</t>
   </si>
   <si>
-    <t xml:space="preserve">* Cimer — Paradise City's upscale spa &amp; water park
+    <t>* Cimer — Paradise City's upscale spa &amp; water park
 * European art-spa aesthetics + pool party + Korean-style sauna (jjimjilbang)
 * Slides, infinity pool; 6-hour pass; seasonal pricing</t>
   </si>
@@ -3824,7 +3828,7 @@
     <t>Water Leisure Day Package</t>
   </si>
   <si>
-    <t xml:space="preserve">* 1-day pass: unlimited water park access + 1-time jet boat ride
+    <t>* 1-day pass: unlimited water park access + 1-time jet boat ride
 * Water skiing, wakeboarding, towable rides, slides, and unlimited BBQ included</t>
   </si>
   <si>
@@ -3846,7 +3850,7 @@
     <t>Water Leisure Afternoon Package</t>
   </si>
   <si>
-    <t xml:space="preserve">* Afternoon pass: water park access + 1-time jet boat ride
+    <t>* Afternoon pass: water park access + 1-time jet boat ride
 * Water skiing, wakeboarding, towable rides, slides, and unlimited BBQ included</t>
   </si>
   <si>
@@ -3871,7 +3875,7 @@
     <t>20-Person Skybox</t>
   </si>
   <si>
-    <t xml:space="preserve">* VIP Skybox at Gocheok Sky Dome for Kiwoom Heroes games
+    <t>* VIP Skybox at Gocheok Sky Dome for Kiwoom Heroes games
 * Dedicated entrance via Central C Gate, private parking, mascot photo service</t>
   </si>
   <si>
@@ -3905,7 +3909,7 @@
     <t>Weekday Skybox</t>
   </si>
   <si>
-    <t xml:space="preserve">* VIP Skybox at Incheon SSG Landers Field for SSG Landers games
+    <t>* VIP Skybox at Incheon SSG Landers Field for SSG Landers games
 * Premium private skybox seating; food and beverages available in-seat</t>
   </si>
   <si>
@@ -3933,7 +3937,7 @@
     <t>Soccer Skybox (FC Seoul)</t>
   </si>
   <si>
-    <t xml:space="preserve">* VIP Skybox at Seoul World Cup Stadium for FC Seoul matches
+    <t>* VIP Skybox at Seoul World Cup Stadium for FC Seoul matches
 * Private skybox with premium stadium views and in-seat dining service</t>
   </si>
   <si>
@@ -3961,7 +3965,7 @@
     <t>5-Ride Magic Pass</t>
   </si>
   <si>
-    <t xml:space="preserve">* 1-Day Pass to Lotte World (indoor + outdoor) with Magic Pass for priority attraction access
+    <t>* 1-Day Pass to Lotte World (indoor + outdoor) with Magic Pass for priority attraction access
 * 5-ride or 7-ride Magic Pass options; no queuing at priority attractions</t>
   </si>
   <si>
@@ -3986,13 +3990,13 @@
     <t>Everland Dream Tour</t>
   </si>
   <si>
-    <t xml:space="preserve">* Everland Dream Tour — VIP guided park experience with full priority access
+    <t>* Everland Dream Tour — VIP guided park experience with full priority access
 * Dedicated parking, front gate priority entry, private guide throughout the park
 * Priority boarding at all major attractions; commemorative photo; restaurant meal included
 * Safari Special Tour (subject to availability)</t>
   </si>
   <si>
-    <t xml:space="preserve">* VIP Everland experience with personal guide, priority access, and restaurant dining
+    <t>* VIP Everland experience with personal guide, priority access, and restaurant dining
 * No waiting in queues — dedicated guide escorts through all major attractions</t>
   </si>
   <si>
@@ -4008,7 +4012,7 @@
     <t>Seoul Land 1-Day Pass</t>
   </si>
   <si>
-    <t xml:space="preserve">* Full-day access to Seoul Land amusement park in Gwacheon
+    <t>* Full-day access to Seoul Land amusement park in Gwacheon
 * Classic Korean theme park with rides, attractions, and family entertainment</t>
   </si>
   <si>
@@ -4033,14 +4037,14 @@
     <t>K-POP CAMP · Basic</t>
   </si>
   <si>
-    <t xml:space="preserve">* Group K-POP basic training (vocal &amp; dance fundamentals)
+    <t>* Group K-POP basic training (vocal &amp; dance fundamentals)
 * K-POP idol hair &amp; makeup styling
 * Premium studio profile photo shoot
 * Short-form (Reels/Shorts) challenge video production
 * Official completion certificate issued</t>
   </si>
   <si>
-    <t xml:space="preserve">* Premium residence accommodation and small-group K-POP experience
+    <t>* Premium residence accommodation and small-group K-POP experience
 * Professional video production team, trending short-form content creation
 * Halal/vegan catering, ISO-certified dance &amp; vocal courses
 * Dedicated instructor, staff, and simultaneous interpretation guide</t>
@@ -4055,7 +4059,7 @@
     <t>K-POP CAMP · Gold</t>
   </si>
   <si>
-    <t xml:space="preserve">* Small-group intensive K-POP training (vocal, dance, stage performance)
+    <t>* Small-group intensive K-POP training (vocal, dance, stage performance)
 * Premium idol styling (stage costume fitting available on request)
 * Individual concept photo shoot (album-style)
 * Professional studio music recording session
@@ -4070,7 +4074,7 @@
     <t>K-POP CAMP · Platinum</t>
   </si>
   <si>
-    <t xml:space="preserve">* 1:1 master training with dedicated vocal/dance director
+    <t>* 1:1 master training with dedicated vocal/dance director
 * VVIP dedicated styling and custom stage design
 * Solo original track production &amp; recording
 * Full-length solo music video (MV) production
@@ -4691,7 +4695,7 @@
     <t>Arabic-Korean Interpretation</t>
   </si>
   <si>
-    <t xml:space="preserve">* Professional Arabic-Korean simultaneous and consecutive interpretation
+    <t>* Professional Arabic-Korean simultaneous and consecutive interpretation
 * Specialized in medical, business, and VIP tourism settings
 * Based in Seoul; available nationwide</t>
   </si>
@@ -4723,7 +4727,7 @@
     <t>General · 8h</t>
   </si>
   <si>
-    <t xml:space="preserve">* Professional Arabic-Korean interpretation (General or Senior/Professional level)
+    <t>* Professional Arabic-Korean interpretation (General or Senior/Professional level)
 * 8-hour daily rate; overtime billed separately
 * Experienced with VIP clients, medical consultations, and high-profile engagements</t>
   </si>
@@ -4755,13 +4759,13 @@
     <t>Noble Klasse Solati S11</t>
   </si>
   <si>
-    <t xml:space="preserve">* Noble Klasse Solati S11 — world's first halal-certified limousine in Korea
+    <t>* Noble Klasse Solati S11 — world's first halal-certified limousine in Korea
 * Dedicated in-vehicle prayer space with qibla direction, prayer mat provided
 * Muslim VIP-optimized mobility service for travel, sightseeing, and medical visits
 * Price on inquiry</t>
   </si>
   <si>
-    <t xml:space="preserve">* World's first halal-certified limousine service in Korea
+    <t>* World's first halal-certified limousine service in Korea
 * In-vehicle prayer space specifically designed for Muslim passengers
 * Enables prayers at any time without stopping — ideal for busy itineraries</t>
   </si>
@@ -4790,7 +4794,7 @@
     <t>Luxury Sedan (Genesis G90) · 8h</t>
   </si>
   <si>
-    <t xml:space="preserve">* 8-hour charter includes driver; base fare covers up to 8h
+    <t>* 8-hour charter includes driver; base fare covers up to 8h
 * Fuel, tolls, parking, and driver meals/accommodation not included
 * English-speaking driver available on request (additional charge)</t>
   </si>
@@ -4843,7 +4847,7 @@
     <t>Luxury Sedan (Genesis G90 RS4) · 10h</t>
   </si>
   <si>
-    <t xml:space="preserve">* 10-hour charter includes driver; all three vehicle types priced equally
+    <t>* 10-hour charter includes driver; all three vehicle types priced equally
 * Latest model fleet: Genesis G90 RS4 / Mercedes S-Class / Mercedes Sprinter VIP
 * Fuel, tolls, parking, and driver meals/accommodation not included</t>
   </si>
@@ -4884,7 +4888,7 @@
     <t>Genesis G90 Long Wheel Limousine · 9h</t>
   </si>
   <si>
-    <t xml:space="preserve">* 9-hour charter (09:00–18:00); overtime billed per hour after 18:00
+    <t>* 9-hour charter (09:00–18:00); overtime billed per hour after 18:00
 * Eligible clients: foreign VIPs/buyers, government bodies, corporate accounts
 * Fuel, tolls, parking, and driver meals/accommodation billed separately</t>
   </si>
@@ -4931,7 +4935,7 @@
     <t>Mercedes-Benz S580L 4MATIC · 8h</t>
   </si>
   <si>
-    <t xml:space="preserve">* 8-hour charter with driver; vehicle-only (24h) also available
+    <t>* 8-hour charter with driver; vehicle-only (24h) also available
 * English-speaking driver: additional surcharge applies
 * 24h vehicle-only option: ₩55,000 own insurance per day
 * Fuel, tolls, driver meals/accommodation billed after the event</t>
@@ -4967,17 +4971,28 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -5018,7 +5033,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -5354,9 +5369,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AD28"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -5385,7 +5400,7 @@
     <col min="30" max="30" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5477,7 +5492,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>30</v>
       </c>
@@ -5569,7 +5584,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>47</v>
       </c>
@@ -5661,7 +5676,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>49</v>
       </c>
@@ -5753,7 +5768,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>52</v>
       </c>
@@ -5845,7 +5860,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>53</v>
       </c>
@@ -5937,7 +5952,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>62</v>
       </c>
@@ -6029,7 +6044,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:30" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>63</v>
       </c>
@@ -6121,7 +6136,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:30" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>65</v>
       </c>
@@ -6213,7 +6228,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>66</v>
       </c>
@@ -6305,7 +6320,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>73</v>
       </c>
@@ -6397,7 +6412,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:30" s="2" customFormat="1" ht="148.5" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>74</v>
       </c>
@@ -6489,7 +6504,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:30" s="2" customFormat="1" ht="148.5" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>77</v>
       </c>
@@ -6581,7 +6596,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>78</v>
       </c>
@@ -6673,7 +6688,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>81</v>
       </c>
@@ -6765,7 +6780,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:30" s="2" customFormat="1" ht="181.5" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>82</v>
       </c>
@@ -6857,7 +6872,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:30" s="2" customFormat="1" ht="181.5" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>90</v>
       </c>
@@ -6949,7 +6964,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:30" s="2" customFormat="1" ht="181.5" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>91</v>
       </c>
@@ -7041,7 +7056,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:30" s="2" customFormat="1" ht="181.5" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>94</v>
       </c>
@@ -7133,7 +7148,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:30" s="2" customFormat="1" ht="409.5" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>95</v>
       </c>
@@ -7225,7 +7240,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:30" s="2" customFormat="1" ht="409.5" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>97</v>
       </c>
@@ -7292,12 +7307,6 @@
       <c r="V21" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W21" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X21" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y21" s="2" t="s">
         <v>44</v>
       </c>
@@ -7317,7 +7326,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:30" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>98</v>
       </c>
@@ -7384,12 +7393,6 @@
       <c r="V22" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W22" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="X22" s="2" t="s">
-        <v>108</v>
-      </c>
       <c r="Y22" s="2" t="s">
         <v>44</v>
       </c>
@@ -7409,7 +7412,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>109</v>
       </c>
@@ -7476,12 +7479,6 @@
       <c r="V23" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W23" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="X23" s="2" t="s">
-        <v>108</v>
-      </c>
       <c r="Y23" s="2" t="s">
         <v>44</v>
       </c>
@@ -7501,7 +7498,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>112</v>
       </c>
@@ -7568,12 +7565,6 @@
       <c r="V24" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W24" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="X24" s="2" t="s">
-        <v>108</v>
-      </c>
       <c r="Y24" s="2" t="s">
         <v>44</v>
       </c>
@@ -7593,7 +7584,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="25" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>115</v>
       </c>
@@ -7660,12 +7651,6 @@
       <c r="V25" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W25" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="X25" s="2" t="s">
-        <v>108</v>
-      </c>
       <c r="Y25" s="2" t="s">
         <v>44</v>
       </c>
@@ -7685,7 +7670,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="26" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>126</v>
       </c>
@@ -7752,12 +7737,6 @@
       <c r="V26" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W26" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="X26" s="2" t="s">
-        <v>108</v>
-      </c>
       <c r="Y26" s="2" t="s">
         <v>44</v>
       </c>
@@ -7777,7 +7756,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="27" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>129</v>
       </c>
@@ -7844,12 +7823,6 @@
       <c r="V27" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W27" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="X27" s="2" t="s">
-        <v>108</v>
-      </c>
       <c r="Y27" s="2" t="s">
         <v>44</v>
       </c>
@@ -7869,7 +7842,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="28" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>134</v>
       </c>
@@ -7936,12 +7909,6 @@
       <c r="V28" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W28" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="X28" s="2" t="s">
-        <v>108</v>
-      </c>
       <c r="Y28" s="2" t="s">
         <v>44</v>
       </c>
@@ -7962,15 +7929,16 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AD181"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -7999,7 +7967,7 @@
     <col min="30" max="30" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8091,7 +8059,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>138</v>
       </c>
@@ -8183,7 +8151,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>149</v>
       </c>
@@ -8275,7 +8243,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>160</v>
       </c>
@@ -8367,7 +8335,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>164</v>
       </c>
@@ -8459,7 +8427,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>168</v>
       </c>
@@ -8551,7 +8519,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>172</v>
       </c>
@@ -8643,7 +8611,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>179</v>
       </c>
@@ -8735,7 +8703,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>182</v>
       </c>
@@ -8827,7 +8795,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>184</v>
       </c>
@@ -8919,7 +8887,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>187</v>
       </c>
@@ -9011,7 +8979,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>191</v>
       </c>
@@ -9103,7 +9071,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>194</v>
       </c>
@@ -9195,7 +9163,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>199</v>
       </c>
@@ -9287,7 +9255,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>202</v>
       </c>
@@ -9379,7 +9347,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>205</v>
       </c>
@@ -9471,7 +9439,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>214</v>
       </c>
@@ -9563,7 +9531,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>217</v>
       </c>
@@ -9655,7 +9623,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>220</v>
       </c>
@@ -9747,7 +9715,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>223</v>
       </c>
@@ -9839,7 +9807,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:30" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>231</v>
       </c>
@@ -9931,7 +9899,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:30" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>234</v>
       </c>
@@ -10023,7 +9991,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>237</v>
       </c>
@@ -10115,7 +10083,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>245</v>
       </c>
@@ -10207,7 +10175,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="25" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>248</v>
       </c>
@@ -10299,7 +10267,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>251</v>
       </c>
@@ -10391,7 +10359,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="27" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>256</v>
       </c>
@@ -10483,7 +10451,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="28" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>259</v>
       </c>
@@ -10575,7 +10543,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="29" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>262</v>
       </c>
@@ -10667,7 +10635,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="30" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>265</v>
       </c>
@@ -10759,7 +10727,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="31" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>268</v>
       </c>
@@ -10851,7 +10819,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="32" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>271</v>
       </c>
@@ -10943,7 +10911,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="33" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>274</v>
       </c>
@@ -11035,7 +11003,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>277</v>
       </c>
@@ -11127,7 +11095,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>280</v>
       </c>
@@ -11219,7 +11187,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="36" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>285</v>
       </c>
@@ -11311,7 +11279,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="37" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>288</v>
       </c>
@@ -11403,7 +11371,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="38" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>291</v>
       </c>
@@ -11495,7 +11463,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="39" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>294</v>
       </c>
@@ -11587,7 +11555,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>298</v>
       </c>
@@ -11679,7 +11647,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>303</v>
       </c>
@@ -11771,7 +11739,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="42" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>306</v>
       </c>
@@ -11863,7 +11831,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="43" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>309</v>
       </c>
@@ -11955,7 +11923,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="44" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>313</v>
       </c>
@@ -12047,7 +12015,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="45" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>316</v>
       </c>
@@ -12139,7 +12107,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="46" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>319</v>
       </c>
@@ -12231,7 +12199,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="47" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>324</v>
       </c>
@@ -12323,7 +12291,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="48" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>327</v>
       </c>
@@ -12415,7 +12383,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="49" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>330</v>
       </c>
@@ -12507,7 +12475,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="50" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>336</v>
       </c>
@@ -12599,7 +12567,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="51" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>339</v>
       </c>
@@ -12691,7 +12659,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="52" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>342</v>
       </c>
@@ -12783,7 +12751,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="53" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>347</v>
       </c>
@@ -12875,7 +12843,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="54" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>351</v>
       </c>
@@ -12967,7 +12935,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="55" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>356</v>
       </c>
@@ -13059,7 +13027,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="56" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>359</v>
       </c>
@@ -13151,7 +13119,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="57" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>364</v>
       </c>
@@ -13243,7 +13211,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="58" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>367</v>
       </c>
@@ -13335,7 +13303,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="59" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>370</v>
       </c>
@@ -13427,7 +13395,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="60" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>376</v>
       </c>
@@ -13519,7 +13487,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="61" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>379</v>
       </c>
@@ -13611,7 +13579,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="62" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>382</v>
       </c>
@@ -13703,7 +13671,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="63" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>388</v>
       </c>
@@ -13795,7 +13763,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="64" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>391</v>
       </c>
@@ -13887,7 +13855,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="65" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>394</v>
       </c>
@@ -13979,7 +13947,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="66" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>397</v>
       </c>
@@ -14071,7 +14039,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="67" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>401</v>
       </c>
@@ -14163,7 +14131,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="68" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>404</v>
       </c>
@@ -14255,7 +14223,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="69" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>409</v>
       </c>
@@ -14347,7 +14315,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="70" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>412</v>
       </c>
@@ -14439,7 +14407,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="71" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>417</v>
       </c>
@@ -14531,7 +14499,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="72" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>421</v>
       </c>
@@ -14623,7 +14591,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="73" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>424</v>
       </c>
@@ -14715,7 +14683,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="74" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>428</v>
       </c>
@@ -14807,7 +14775,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="75" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>433</v>
       </c>
@@ -14899,7 +14867,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="76" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>439</v>
       </c>
@@ -14991,7 +14959,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="77" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>445</v>
       </c>
@@ -15083,7 +15051,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="78" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>450</v>
       </c>
@@ -15175,7 +15143,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="79" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>456</v>
       </c>
@@ -15267,7 +15235,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="80" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
         <v>459</v>
       </c>
@@ -15359,7 +15327,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="81" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>464</v>
       </c>
@@ -15451,7 +15419,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="82" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>469</v>
       </c>
@@ -15543,7 +15511,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="83" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
         <v>475</v>
       </c>
@@ -15635,7 +15603,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="84" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
         <v>482</v>
       </c>
@@ -15727,7 +15695,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="85" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>488</v>
       </c>
@@ -15819,7 +15787,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="86" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
         <v>494</v>
       </c>
@@ -15911,7 +15879,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="87" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
         <v>499</v>
       </c>
@@ -16003,7 +15971,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="88" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
         <v>504</v>
       </c>
@@ -16095,7 +16063,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="89" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
         <v>509</v>
       </c>
@@ -16187,7 +16155,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="90" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>515</v>
       </c>
@@ -16279,7 +16247,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="91" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
         <v>521</v>
       </c>
@@ -16371,7 +16339,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="92" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
         <v>525</v>
       </c>
@@ -16463,7 +16431,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="93" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
         <v>528</v>
       </c>
@@ -16555,7 +16523,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="94" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
         <v>531</v>
       </c>
@@ -16647,7 +16615,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="95" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
         <v>534</v>
       </c>
@@ -16739,7 +16707,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="96" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
         <v>539</v>
       </c>
@@ -16831,7 +16799,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="97" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
         <v>542</v>
       </c>
@@ -16923,7 +16891,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="98" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
         <v>544</v>
       </c>
@@ -17015,7 +16983,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="99" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
         <v>548</v>
       </c>
@@ -17107,7 +17075,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="100" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
         <v>552</v>
       </c>
@@ -17199,7 +17167,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="101" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
         <v>555</v>
       </c>
@@ -17291,7 +17259,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="102" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
         <v>560</v>
       </c>
@@ -17383,7 +17351,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="103" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
         <v>565</v>
       </c>
@@ -17475,7 +17443,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="104" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
         <v>568</v>
       </c>
@@ -17567,7 +17535,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="105" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
         <v>573</v>
       </c>
@@ -17659,7 +17627,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="106" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
         <v>578</v>
       </c>
@@ -17751,7 +17719,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="107" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
         <v>582</v>
       </c>
@@ -17843,7 +17811,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="108" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
         <v>585</v>
       </c>
@@ -17935,7 +17903,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="109" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
         <v>589</v>
       </c>
@@ -18027,7 +17995,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="110" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
         <v>592</v>
       </c>
@@ -18119,7 +18087,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="111" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
         <v>596</v>
       </c>
@@ -18211,7 +18179,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="112" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
         <v>601</v>
       </c>
@@ -18303,7 +18271,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="113" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A113" s="2" t="s">
         <v>606</v>
       </c>
@@ -18395,7 +18363,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="114" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A114" s="2" t="s">
         <v>611</v>
       </c>
@@ -18487,7 +18455,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="115" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A115" s="2" t="s">
         <v>614</v>
       </c>
@@ -18579,7 +18547,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="116" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A116" s="2" t="s">
         <v>619</v>
       </c>
@@ -18671,7 +18639,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="117" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A117" s="2" t="s">
         <v>625</v>
       </c>
@@ -18763,7 +18731,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="118" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A118" s="2" t="s">
         <v>629</v>
       </c>
@@ -18855,7 +18823,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="119" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A119" s="2" t="s">
         <v>634</v>
       </c>
@@ -18947,7 +18915,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="120" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A120" s="2" t="s">
         <v>638</v>
       </c>
@@ -19039,7 +19007,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="121" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A121" s="2" t="s">
         <v>642</v>
       </c>
@@ -19131,7 +19099,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="122" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A122" s="2" t="s">
         <v>646</v>
       </c>
@@ -19223,7 +19191,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="123" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A123" s="2" t="s">
         <v>649</v>
       </c>
@@ -19315,7 +19283,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="124" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A124" s="2" t="s">
         <v>653</v>
       </c>
@@ -19407,7 +19375,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="125" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A125" s="2" t="s">
         <v>656</v>
       </c>
@@ -19499,7 +19467,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="126" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A126" s="2" t="s">
         <v>660</v>
       </c>
@@ -19591,7 +19559,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="127" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A127" s="2" t="s">
         <v>665</v>
       </c>
@@ -19658,12 +19626,6 @@
       <c r="V127" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W127" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X127" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y127" s="2" t="s">
         <v>44</v>
       </c>
@@ -19683,7 +19645,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="128" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A128" s="2" t="s">
         <v>669</v>
       </c>
@@ -19750,12 +19712,6 @@
       <c r="V128" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W128" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X128" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y128" s="2" t="s">
         <v>44</v>
       </c>
@@ -19775,7 +19731,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="129" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A129" s="2" t="s">
         <v>674</v>
       </c>
@@ -19842,12 +19798,6 @@
       <c r="V129" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W129" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X129" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y129" s="2" t="s">
         <v>44</v>
       </c>
@@ -19867,7 +19817,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="130" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A130" s="2" t="s">
         <v>677</v>
       </c>
@@ -19934,12 +19884,6 @@
       <c r="V130" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W130" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X130" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y130" s="2" t="s">
         <v>44</v>
       </c>
@@ -19959,7 +19903,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="131" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A131" s="2" t="s">
         <v>680</v>
       </c>
@@ -20026,12 +19970,6 @@
       <c r="V131" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W131" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X131" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y131" s="2" t="s">
         <v>44</v>
       </c>
@@ -20051,7 +19989,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="132" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A132" s="2" t="s">
         <v>683</v>
       </c>
@@ -20118,12 +20056,6 @@
       <c r="V132" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W132" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X132" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y132" s="2" t="s">
         <v>44</v>
       </c>
@@ -20143,7 +20075,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="133" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A133" s="2" t="s">
         <v>686</v>
       </c>
@@ -20210,12 +20142,6 @@
       <c r="V133" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W133" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X133" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="Y133" s="2" t="s">
         <v>44</v>
       </c>
@@ -20235,7 +20161,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="134" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A134" s="2" t="s">
         <v>690</v>
       </c>
@@ -20302,12 +20228,6 @@
       <c r="V134" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W134" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X134" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="Y134" s="2" t="s">
         <v>44</v>
       </c>
@@ -20327,7 +20247,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="135" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A135" s="2" t="s">
         <v>694</v>
       </c>
@@ -20394,12 +20314,6 @@
       <c r="V135" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W135" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X135" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="Y135" s="2" t="s">
         <v>44</v>
       </c>
@@ -20419,7 +20333,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="136" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A136" s="2" t="s">
         <v>697</v>
       </c>
@@ -20486,12 +20400,6 @@
       <c r="V136" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W136" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X136" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="Y136" s="2" t="s">
         <v>44</v>
       </c>
@@ -20511,7 +20419,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="137" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A137" s="2" t="s">
         <v>702</v>
       </c>
@@ -20578,12 +20486,6 @@
       <c r="V137" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W137" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X137" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="Y137" s="2" t="s">
         <v>44</v>
       </c>
@@ -20603,7 +20505,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="138" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A138" s="2" t="s">
         <v>705</v>
       </c>
@@ -20670,12 +20572,6 @@
       <c r="V138" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W138" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X138" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="Y138" s="2" t="s">
         <v>44</v>
       </c>
@@ -20695,7 +20591,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="139" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A139" s="2" t="s">
         <v>708</v>
       </c>
@@ -20762,12 +20658,6 @@
       <c r="V139" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W139" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X139" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="Y139" s="2" t="s">
         <v>44</v>
       </c>
@@ -20787,7 +20677,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="140" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A140" s="2" t="s">
         <v>711</v>
       </c>
@@ -20854,12 +20744,6 @@
       <c r="V140" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W140" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X140" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="Y140" s="2" t="s">
         <v>44</v>
       </c>
@@ -20879,7 +20763,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="141" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A141" s="2" t="s">
         <v>714</v>
       </c>
@@ -20946,12 +20830,6 @@
       <c r="V141" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W141" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X141" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y141" s="2" t="s">
         <v>44</v>
       </c>
@@ -20971,7 +20849,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="142" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A142" s="2" t="s">
         <v>717</v>
       </c>
@@ -21038,12 +20916,6 @@
       <c r="V142" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W142" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X142" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y142" s="2" t="s">
         <v>44</v>
       </c>
@@ -21063,7 +20935,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="143" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A143" s="2" t="s">
         <v>720</v>
       </c>
@@ -21130,12 +21002,6 @@
       <c r="V143" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W143" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X143" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y143" s="2" t="s">
         <v>44</v>
       </c>
@@ -21155,7 +21021,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="144" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A144" s="2" t="s">
         <v>723</v>
       </c>
@@ -21222,12 +21088,6 @@
       <c r="V144" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W144" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X144" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y144" s="2" t="s">
         <v>44</v>
       </c>
@@ -21247,7 +21107,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="145" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A145" s="2" t="s">
         <v>726</v>
       </c>
@@ -21314,12 +21174,6 @@
       <c r="V145" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W145" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X145" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y145" s="2" t="s">
         <v>44</v>
       </c>
@@ -21339,7 +21193,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="146" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A146" s="2" t="s">
         <v>729</v>
       </c>
@@ -21406,12 +21260,6 @@
       <c r="V146" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W146" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X146" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y146" s="2" t="s">
         <v>44</v>
       </c>
@@ -21431,7 +21279,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="147" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A147" s="2" t="s">
         <v>733</v>
       </c>
@@ -21498,12 +21346,6 @@
       <c r="V147" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W147" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X147" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y147" s="2" t="s">
         <v>44</v>
       </c>
@@ -21523,7 +21365,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="148" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A148" s="2" t="s">
         <v>736</v>
       </c>
@@ -21590,12 +21432,6 @@
       <c r="V148" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W148" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X148" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y148" s="2" t="s">
         <v>44</v>
       </c>
@@ -21615,7 +21451,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="149" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A149" s="2" t="s">
         <v>739</v>
       </c>
@@ -21682,12 +21518,6 @@
       <c r="V149" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W149" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X149" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y149" s="2" t="s">
         <v>44</v>
       </c>
@@ -21707,7 +21537,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="150" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A150" s="2" t="s">
         <v>742</v>
       </c>
@@ -21774,12 +21604,6 @@
       <c r="V150" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W150" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X150" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y150" s="2" t="s">
         <v>44</v>
       </c>
@@ -21799,7 +21623,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="151" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A151" s="2" t="s">
         <v>745</v>
       </c>
@@ -21866,12 +21690,6 @@
       <c r="V151" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W151" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X151" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y151" s="2" t="s">
         <v>44</v>
       </c>
@@ -21891,7 +21709,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="152" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A152" s="2" t="s">
         <v>748</v>
       </c>
@@ -21958,12 +21776,6 @@
       <c r="V152" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W152" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X152" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y152" s="2" t="s">
         <v>44</v>
       </c>
@@ -21983,7 +21795,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="153" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A153" s="2" t="s">
         <v>753</v>
       </c>
@@ -22050,12 +21862,6 @@
       <c r="V153" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W153" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X153" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y153" s="2" t="s">
         <v>44</v>
       </c>
@@ -22075,7 +21881,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="154" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A154" s="2" t="s">
         <v>756</v>
       </c>
@@ -22142,12 +21948,6 @@
       <c r="V154" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W154" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X154" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y154" s="2" t="s">
         <v>44</v>
       </c>
@@ -22167,7 +21967,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="155" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A155" s="2" t="s">
         <v>759</v>
       </c>
@@ -22234,12 +22034,6 @@
       <c r="V155" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W155" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X155" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y155" s="2" t="s">
         <v>44</v>
       </c>
@@ -22259,7 +22053,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="156" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A156" s="2" t="s">
         <v>762</v>
       </c>
@@ -22326,12 +22120,6 @@
       <c r="V156" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W156" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X156" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y156" s="2" t="s">
         <v>44</v>
       </c>
@@ -22351,7 +22139,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="157" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A157" s="2" t="s">
         <v>765</v>
       </c>
@@ -22418,12 +22206,6 @@
       <c r="V157" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W157" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X157" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y157" s="2" t="s">
         <v>44</v>
       </c>
@@ -22443,7 +22225,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="158" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A158" s="2" t="s">
         <v>768</v>
       </c>
@@ -22510,12 +22292,6 @@
       <c r="V158" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W158" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X158" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y158" s="2" t="s">
         <v>44</v>
       </c>
@@ -22535,7 +22311,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="159" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A159" s="2" t="s">
         <v>771</v>
       </c>
@@ -22602,12 +22378,6 @@
       <c r="V159" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W159" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X159" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y159" s="2" t="s">
         <v>44</v>
       </c>
@@ -22627,7 +22397,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="160" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A160" s="2" t="s">
         <v>774</v>
       </c>
@@ -22694,12 +22464,6 @@
       <c r="V160" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W160" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X160" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y160" s="2" t="s">
         <v>44</v>
       </c>
@@ -22719,7 +22483,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="161" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A161" s="2" t="s">
         <v>777</v>
       </c>
@@ -22786,12 +22550,6 @@
       <c r="V161" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W161" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X161" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y161" s="2" t="s">
         <v>44</v>
       </c>
@@ -22811,7 +22569,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="162" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A162" s="2" t="s">
         <v>780</v>
       </c>
@@ -22878,12 +22636,6 @@
       <c r="V162" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W162" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X162" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y162" s="2" t="s">
         <v>44</v>
       </c>
@@ -22903,7 +22655,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="163" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A163" s="2" t="s">
         <v>783</v>
       </c>
@@ -22970,12 +22722,6 @@
       <c r="V163" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W163" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X163" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y163" s="2" t="s">
         <v>44</v>
       </c>
@@ -22995,7 +22741,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="164" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A164" s="2" t="s">
         <v>786</v>
       </c>
@@ -23062,12 +22808,6 @@
       <c r="V164" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W164" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X164" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y164" s="2" t="s">
         <v>44</v>
       </c>
@@ -23087,7 +22827,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="165" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A165" s="2" t="s">
         <v>789</v>
       </c>
@@ -23154,12 +22894,6 @@
       <c r="V165" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W165" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X165" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y165" s="2" t="s">
         <v>44</v>
       </c>
@@ -23179,7 +22913,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="166" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A166" s="2" t="s">
         <v>792</v>
       </c>
@@ -23246,12 +22980,6 @@
       <c r="V166" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W166" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X166" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y166" s="2" t="s">
         <v>44</v>
       </c>
@@ -23271,7 +22999,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="167" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A167" s="2" t="s">
         <v>795</v>
       </c>
@@ -23363,7 +23091,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="168" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A168" s="2" t="s">
         <v>798</v>
       </c>
@@ -23455,7 +23183,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="169" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A169" s="2" t="s">
         <v>801</v>
       </c>
@@ -23547,7 +23275,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="170" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A170" s="2" t="s">
         <v>804</v>
       </c>
@@ -23639,7 +23367,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="171" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A171" s="2" t="s">
         <v>807</v>
       </c>
@@ -23731,7 +23459,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="172" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A172" s="2" t="s">
         <v>810</v>
       </c>
@@ -23823,7 +23551,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="173" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A173" s="2" t="s">
         <v>813</v>
       </c>
@@ -23915,7 +23643,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="174" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A174" s="2" t="s">
         <v>816</v>
       </c>
@@ -24007,7 +23735,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="175" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A175" s="2" t="s">
         <v>819</v>
       </c>
@@ -24099,7 +23827,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="176" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A176" s="2" t="s">
         <v>822</v>
       </c>
@@ -24191,7 +23919,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="177" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A177" s="2" t="s">
         <v>825</v>
       </c>
@@ -24283,7 +24011,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="178" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A178" s="2" t="s">
         <v>828</v>
       </c>
@@ -24375,7 +24103,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="179" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A179" s="2" t="s">
         <v>831</v>
       </c>
@@ -24467,7 +24195,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="180" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A180" s="2" t="s">
         <v>834</v>
       </c>
@@ -24559,7 +24287,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="181" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A181" s="2" t="s">
         <v>837</v>
       </c>
@@ -24652,15 +24380,16 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AD77"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -24689,7 +24418,7 @@
     <col min="30" max="30" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -24781,7 +24510,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>840</v>
       </c>
@@ -24873,7 +24602,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>849</v>
       </c>
@@ -24965,7 +24694,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>857</v>
       </c>
@@ -25057,7 +24786,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>859</v>
       </c>
@@ -25149,7 +24878,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>862</v>
       </c>
@@ -25241,7 +24970,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>865</v>
       </c>
@@ -25333,7 +25062,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>868</v>
       </c>
@@ -25425,7 +25154,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>874</v>
       </c>
@@ -25517,7 +25246,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>877</v>
       </c>
@@ -25609,7 +25338,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>880</v>
       </c>
@@ -25701,7 +25430,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>887</v>
       </c>
@@ -25793,7 +25522,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>890</v>
       </c>
@@ -25885,7 +25614,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>894</v>
       </c>
@@ -25977,7 +25706,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>898</v>
       </c>
@@ -26069,7 +25798,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>902</v>
       </c>
@@ -26161,7 +25890,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>905</v>
       </c>
@@ -26253,7 +25982,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>908</v>
       </c>
@@ -26345,7 +26074,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>911</v>
       </c>
@@ -26437,7 +26166,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>914</v>
       </c>
@@ -26529,7 +26258,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>917</v>
       </c>
@@ -26621,7 +26350,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>924</v>
       </c>
@@ -26713,7 +26442,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:30" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>934</v>
       </c>
@@ -26805,7 +26534,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>943</v>
       </c>
@@ -26897,7 +26626,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="25" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>951</v>
       </c>
@@ -26989,7 +26718,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>958</v>
       </c>
@@ -27081,7 +26810,7 @@
         <v>968</v>
       </c>
     </row>
-    <row r="27" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>969</v>
       </c>
@@ -27173,7 +26902,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="28" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>976</v>
       </c>
@@ -27265,7 +26994,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="29" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:30" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>983</v>
       </c>
@@ -27357,7 +27086,7 @@
         <v>968</v>
       </c>
     </row>
-    <row r="30" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>988</v>
       </c>
@@ -27449,7 +27178,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="31" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>995</v>
       </c>
@@ -27541,7 +27270,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="32" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>1001</v>
       </c>
@@ -27633,7 +27362,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="33" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>1009</v>
       </c>
@@ -27725,7 +27454,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>1016</v>
       </c>
@@ -27817,7 +27546,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>1018</v>
       </c>
@@ -27909,7 +27638,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="36" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>1024</v>
       </c>
@@ -28001,7 +27730,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="37" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>1030</v>
       </c>
@@ -28093,7 +27822,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="38" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>1037</v>
       </c>
@@ -28185,7 +27914,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="39" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>1044</v>
       </c>
@@ -28277,7 +28006,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>1050</v>
       </c>
@@ -28369,7 +28098,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>1056</v>
       </c>
@@ -28461,7 +28190,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="42" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>1065</v>
       </c>
@@ -28528,12 +28257,6 @@
       <c r="V42" s="2" t="s">
         <v>1071</v>
       </c>
-      <c r="W42" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X42" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y42" s="2" t="s">
         <v>44</v>
       </c>
@@ -28553,7 +28276,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="43" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:30" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>1073</v>
       </c>
@@ -28620,12 +28343,6 @@
       <c r="V43" s="2" t="s">
         <v>1079</v>
       </c>
-      <c r="W43" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X43" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="Y43" s="2" t="s">
         <v>1080</v>
       </c>
@@ -28645,7 +28362,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="44" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>1081</v>
       </c>
@@ -28712,12 +28429,6 @@
       <c r="V44" s="2" t="s">
         <v>1086</v>
       </c>
-      <c r="W44" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X44" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="Y44" s="2" t="s">
         <v>44</v>
       </c>
@@ -28737,7 +28448,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="45" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>1088</v>
       </c>
@@ -28804,12 +28515,6 @@
       <c r="V45" s="2" t="s">
         <v>1093</v>
       </c>
-      <c r="W45" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X45" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="Y45" s="2" t="s">
         <v>1080</v>
       </c>
@@ -28829,7 +28534,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="46" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:30" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>1094</v>
       </c>
@@ -28921,7 +28626,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="47" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>1102</v>
       </c>
@@ -29013,7 +28718,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="48" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>1108</v>
       </c>
@@ -29105,7 +28810,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="49" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>1117</v>
       </c>
@@ -29197,7 +28902,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="50" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>1125</v>
       </c>
@@ -29289,7 +28994,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="51" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>1133</v>
       </c>
@@ -29381,7 +29086,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="52" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>1145</v>
       </c>
@@ -29473,7 +29178,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="53" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>1148</v>
       </c>
@@ -29565,7 +29270,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="54" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>1157</v>
       </c>
@@ -29657,7 +29362,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="55" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>1159</v>
       </c>
@@ -29749,7 +29454,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="56" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>1167</v>
       </c>
@@ -29841,7 +29546,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="57" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>1169</v>
       </c>
@@ -29933,7 +29638,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="58" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>1176</v>
       </c>
@@ -30025,7 +29730,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="59" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>1177</v>
       </c>
@@ -30117,7 +29822,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="60" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>1185</v>
       </c>
@@ -30209,7 +29914,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="61" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>1187</v>
       </c>
@@ -30301,7 +30006,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="62" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>1189</v>
       </c>
@@ -30393,7 +30098,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="63" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>1196</v>
       </c>
@@ -30485,7 +30190,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="64" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>1198</v>
       </c>
@@ -30577,7 +30282,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="65" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>1200</v>
       </c>
@@ -30669,7 +30374,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="66" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>1208</v>
       </c>
@@ -30761,7 +30466,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="67" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>1210</v>
       </c>
@@ -30853,7 +30558,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="68" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>1218</v>
       </c>
@@ -30945,7 +30650,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="69" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>1224</v>
       </c>
@@ -31037,7 +30742,7 @@
         <v>1233</v>
       </c>
     </row>
-    <row r="70" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>1234</v>
       </c>
@@ -31129,7 +30834,7 @@
         <v>1233</v>
       </c>
     </row>
-    <row r="71" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>1236</v>
       </c>
@@ -31221,7 +30926,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="72" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>1244</v>
       </c>
@@ -31313,7 +31018,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="73" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>1246</v>
       </c>
@@ -31405,7 +31110,7 @@
         <v>1233</v>
       </c>
     </row>
-    <row r="74" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>1253</v>
       </c>
@@ -31497,7 +31202,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="75" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>1260</v>
       </c>
@@ -31589,7 +31294,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="76" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:30" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>1262</v>
       </c>
@@ -31681,7 +31386,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="77" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>1269</v>
       </c>
@@ -31774,15 +31479,16 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:AD4"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -31811,7 +31517,7 @@
     <col min="30" max="30" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -31903,7 +31609,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1275</v>
       </c>
@@ -31970,12 +31676,6 @@
       <c r="V2" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X2" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="Y2" s="2" t="s">
         <v>1080</v>
       </c>
@@ -31995,7 +31695,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>1283</v>
       </c>
@@ -32062,12 +31762,6 @@
       <c r="V3" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W3" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X3" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="Y3" s="2" t="s">
         <v>1080</v>
       </c>
@@ -32087,7 +31781,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>1286</v>
       </c>
@@ -32154,12 +31848,6 @@
       <c r="V4" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="W4" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="X4" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="Y4" s="2" t="s">
         <v>1080</v>
       </c>
@@ -32180,15 +31868,16 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:AD4"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -32217,7 +31906,7 @@
     <col min="30" max="30" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -32309,7 +31998,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" s="2" customFormat="1" ht="148.5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1289</v>
       </c>
@@ -32401,7 +32090,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" s="2" customFormat="1" ht="148.5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>1296</v>
       </c>
@@ -32493,7 +32182,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>1300</v>
       </c>
@@ -32586,15 +32275,16 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:AD63"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -32623,7 +32313,7 @@
     <col min="30" max="30" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -32715,7 +32405,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1303</v>
       </c>
@@ -32807,7 +32497,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>1311</v>
       </c>
@@ -32899,7 +32589,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>1315</v>
       </c>
@@ -32991,7 +32681,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>1321</v>
       </c>
@@ -33083,7 +32773,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>1324</v>
       </c>
@@ -33175,7 +32865,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>1330</v>
       </c>
@@ -33267,7 +32957,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="8" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>1336</v>
       </c>
@@ -33359,7 +33049,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>1340</v>
       </c>
@@ -33451,7 +33141,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>1350</v>
       </c>
@@ -33543,7 +33233,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>1353</v>
       </c>
@@ -33635,7 +33325,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>1356</v>
       </c>
@@ -33727,7 +33417,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>1359</v>
       </c>
@@ -33819,7 +33509,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>1366</v>
       </c>
@@ -33911,7 +33601,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>1369</v>
       </c>
@@ -34003,7 +33693,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>1372</v>
       </c>
@@ -34095,7 +33785,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>1374</v>
       </c>
@@ -34187,7 +33877,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>1381</v>
       </c>
@@ -34279,7 +33969,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>1384</v>
       </c>
@@ -34371,7 +34061,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>1389</v>
       </c>
@@ -34463,7 +34153,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>1392</v>
       </c>
@@ -34555,7 +34245,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>1397</v>
       </c>
@@ -34647,7 +34337,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>1400</v>
       </c>
@@ -34739,7 +34429,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>1403</v>
       </c>
@@ -34831,7 +34521,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="25" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>1410</v>
       </c>
@@ -34923,7 +34613,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>1413</v>
       </c>
@@ -35015,7 +34705,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="27" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>1416</v>
       </c>
@@ -35107,7 +34797,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="28" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>1421</v>
       </c>
@@ -35199,7 +34889,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="29" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>1423</v>
       </c>
@@ -35291,7 +34981,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="30" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>1426</v>
       </c>
@@ -35383,7 +35073,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="31" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>1428</v>
       </c>
@@ -35475,7 +35165,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="32" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>1432</v>
       </c>
@@ -35567,7 +35257,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="33" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>1434</v>
       </c>
@@ -35659,7 +35349,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>1440</v>
       </c>
@@ -35751,7 +35441,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>1443</v>
       </c>
@@ -35843,7 +35533,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="36" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>1446</v>
       </c>
@@ -35935,7 +35625,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="37" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>1451</v>
       </c>
@@ -36027,7 +35717,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="38" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>1456</v>
       </c>
@@ -36119,7 +35809,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="39" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>1466</v>
       </c>
@@ -36211,7 +35901,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="40" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>1469</v>
       </c>
@@ -36303,7 +35993,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="41" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>1472</v>
       </c>
@@ -36395,7 +36085,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="42" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>1476</v>
       </c>
@@ -36487,7 +36177,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="43" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>1479</v>
       </c>
@@ -36579,7 +36269,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="44" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>1483</v>
       </c>
@@ -36671,7 +36361,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="45" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>1486</v>
       </c>
@@ -36763,7 +36453,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="46" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>1489</v>
       </c>
@@ -36855,7 +36545,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="47" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>1497</v>
       </c>
@@ -36947,7 +36637,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="48" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>1500</v>
       </c>
@@ -37039,7 +36729,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="49" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>1506</v>
       </c>
@@ -37131,7 +36821,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="50" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>1508</v>
       </c>
@@ -37223,7 +36913,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="51" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>1518</v>
       </c>
@@ -37315,7 +37005,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="52" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>1529</v>
       </c>
@@ -37407,7 +37097,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="53" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>1532</v>
       </c>
@@ -37499,7 +37189,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="54" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>1535</v>
       </c>
@@ -37591,7 +37281,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="55" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>1537</v>
       </c>
@@ -37683,7 +37373,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="56" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>1545</v>
       </c>
@@ -37775,7 +37465,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="57" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>1547</v>
       </c>
@@ -37867,7 +37557,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="58" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>1549</v>
       </c>
@@ -37959,7 +37649,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="59" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>1559</v>
       </c>
@@ -38051,7 +37741,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="60" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>1562</v>
       </c>
@@ -38143,7 +37833,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="61" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>1564</v>
       </c>
@@ -38235,7 +37925,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="62" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>1572</v>
       </c>
@@ -38327,7 +38017,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="63" spans="1:30" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>1575</v>
       </c>
@@ -38420,7 +38110,8 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>